<commit_message>
feat: replica componente Footer para a página Dashboard (substitui footer simples)
</commit_message>
<xml_diff>
--- a/ORCAMENTOS - PROGRAMAS.xlsx
+++ b/ORCAMENTOS - PROGRAMAS.xlsx
@@ -13,22 +13,23 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={0619dc93-171c-4da2-b441-412af1ac3113}</author>
-    <author>tc={2a7dcfa7-c60f-45b9-842b-040baa35e254}</author>
-    <author>tc={c04e08d9-b3a5-458c-a077-712e51e5ccf6}</author>
-    <author>tc={f06b32da-dd55-4e63-aef3-1f65e72a0c83}</author>
+    <author>tc={3db4590b-99b0-46f9-8e5c-535b09fd0c09}</author>
+    <author>tc={8244c2f2-4132-4074-9ca2-389a2fe912cd}</author>
+    <author>tc={8ba3ea41-de65-44d7-bcaf-e66d12b358bb}</author>
+    <author>tc={bbd46d50-5793-4f27-acbb-bf2b066df97a}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{0619dc93-171c-4da2-b441-412af1ac3113}" ref="A1">
+    <comment authorId="0" xr:uid="{3db4590b-99b0-46f9-8e5c-535b09fd0c09}" ref="A73">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-	@luisalnr@gmail.com manter apenas no Eixo VI - linha 163 da planilha
+	Não apareceram os seguintes órgãos: TCE, TJAC, DPE, MPAC (estão listados na planilha anterior, mas não estão nesta) @luisalnr@gmail.com
+Assigned to luisalnr@gmail.com
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{2a7dcfa7-c60f-45b9-842b-040baa35e254}" ref="E68">
+    <comment authorId="1" xr:uid="{8244c2f2-4132-4074-9ca2-389a2fe912cd}" ref="E68">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -39,17 +40,16 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{c04e08d9-b3a5-458c-a077-712e51e5ccf6}" ref="A73">
+    <comment authorId="2" xr:uid="{8ba3ea41-de65-44d7-bcaf-e66d12b358bb}" ref="A1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-	Não apareceram os seguintes órgãos: TCE, TJAC, DPE, MPAC (estão listados na planilha anterior, mas não estão nesta) @luisalnr@gmail.com
-Assigned to luisalnr@gmail.com
+	@luisalnr@gmail.com manter apenas no Eixo VI - linha 163 da planilha
 </t>
       </text>
     </comment>
-    <comment authorId="3" xr:uid="{f06b32da-dd55-4e63-aef3-1f65e72a0c83}" ref="E73">
+    <comment authorId="3" xr:uid="{bbd46d50-5793-4f27-acbb-bf2b066df97a}" ref="E73">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="273">
   <si>
     <t>Eixo</t>
   </si>
@@ -97,7 +97,7 @@
     <t>18 – Gestão Ambiental</t>
   </si>
   <si>
-    <t>715/199 - SEFAZ</t>
+    <t>715/199 - SEFAZ (Departamento do Tesouro Estadual)</t>
   </si>
   <si>
     <t>PROSPECÇÃO DE MERCADO DA ECONOMIA
@@ -379,9 +379,6 @@
   </si>
   <si>
     <t>CONSTRUÇÃO, REFORMA E AMPLIAÇÃO DOS PRÉDIOS DA PGE.</t>
-  </si>
-  <si>
-    <t>715/199 - SEFAZ (Departamento do Tesouro Estadual)</t>
   </si>
   <si>
     <t>PROGRAMA ESTADUAL DE ENFRENTAMENTO ÀS DEMANDAS CONTINGENTES.</t>
@@ -1007,7 +1004,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="48">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1122,9 +1119,6 @@
     </xf>
     <xf borderId="1" fillId="4" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="4" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right"/>
@@ -1259,22 +1253,22 @@
 
 <file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
 <Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks">
-  <Task id="{b50e36b7-5e74-4168-ae7d-4022b894adff}">
+  <Task id="{7f02e35a-7017-4008-a94e-1ebb9b3b14da}">
     <Anchor>
-      <Comment id="{c04e08d9-b3a5-458c-a077-712e51e5ccf6}"/>
+      <Comment id="{3db4590b-99b0-46f9-8e5c-535b09fd0c09}"/>
     </Anchor>
     <History>
-      <Event time="2026-06-05T13:55:13.00" id="{6aa7667b-d93b-4be4-b33e-5689492c863a}">
+      <Event time="2026-06-05T13:55:13.00" id="{33258cc1-57c5-427e-b0cf-7728908c8532}">
         <Attribution userId="placeholder@email.com" userName="Roseneide Sena" userProvider="google-sheets"/>
         <Anchor>
-          <Comment id="{c04e08d9-b3a5-458c-a077-712e51e5ccf6}"/>
+          <Comment id="{3db4590b-99b0-46f9-8e5c-535b09fd0c09}"/>
         </Anchor>
         <Create/>
       </Event>
-      <Event time="2026-06-05T13:55:13.00" id="{d38ca453-1983-4476-98ee-5aff7b39107e}">
+      <Event time="2026-06-05T13:55:13.00" id="{6e82845f-603e-460e-b6f7-d006793ace38}">
         <Attribution userId="placeholder@email.com" userName="Roseneide Sena" userProvider="google-sheets"/>
         <Anchor>
-          <Comment id="{c04e08d9-b3a5-458c-a077-712e51e5ccf6}"/>
+          <Comment id="{3db4590b-99b0-46f9-8e5c-535b09fd0c09}"/>
         </Anchor>
         <Assign userId="luisalnr@gmail.com" userName="luisalnr@gmail.com" userProvider="google-sheets"/>
       </Event>
@@ -1289,11 +1283,11 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="luisalnr@gmail.com" id="{412111f0-d9ef-41f6-b055-45c4ed45d33c}" userId="luisalnr@gmail.com" providerId="google-sheets"/>
-  <x18tc:person displayName="Roseneide Sena" id="{96b38dae-aaad-4c58-8713-07ba69f8f13c}" providerId="google-sheets"/>
-  <x18tc:person displayName="Vinícius_Oikonomia" id="{96cb20ff-ca75-4803-bcce-b3200dd39887}" providerId="google-sheets"/>
-  <x18tc:person displayName="rsena.acre@gmail.com" id="{2b2a40fd-1d02-433a-97cf-450b5792e745}" userId="rsena.acre@gmail.com" providerId="google-sheets"/>
-  <x18tc:person displayName="Luísa Ribeiro" id="{4a970b55-9de4-44b4-b664-773b73a5c0ca}" providerId="google-sheets"/>
+  <x18tc:person displayName="luisalnr@gmail.com" id="{04d0802d-6b46-4da0-9c28-31ea27299ecf}" userId="luisalnr@gmail.com" providerId="google-sheets"/>
+  <x18tc:person displayName="Roseneide Sena" id="{18a4e096-09dc-487e-94e2-bb4f2bc6690b}" providerId="google-sheets"/>
+  <x18tc:person displayName="Vinícius_Oikonomia" id="{4b7fa688-6db5-404c-a3ea-4ec0609ed5c5}" providerId="google-sheets"/>
+  <x18tc:person displayName="rsena.acre@gmail.com" id="{a4db4c2b-c5e8-4071-a7cd-2df124f7c271}" userId="rsena.acre@gmail.com" providerId="google-sheets"/>
+  <x18tc:person displayName="Luísa Ribeiro" id="{85e82f82-b122-4a5e-827e-e13eb07226b3}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -1633,35 +1627,35 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="E73" dT="2026-06-08T13:15:23.00" personId="{96cb20ff-ca75-4803-bcce-b3200dd39887}" id="{f06b32da-dd55-4e63-aef3-1f65e72a0c83}" done="0">
+  <x18tc:threadedComment ref="E73" dT="2026-06-08T13:15:23.00" personId="{4b7fa688-6db5-404c-a3ea-4ec0609ed5c5}" id="{bbd46d50-5793-4f27-acbb-bf2b066df97a}" done="0">
     <x18tc:text xml:space="preserve">No QDD, consta valor inicial de R$2000, consideramos R$1000 ou R$2000 @rsena.acre@gmail.com</x18tc:text>
     <x18tc:mentions>
-      <x18tc:mention mentionpersonId="{2b2a40fd-1d02-433a-97cf-450b5792e745}" mentionId="{c73ce117-07e8-445d-bb33-afc23e89eae7}" startIndex="70" length="21"/>
+      <x18tc:mention mentionpersonId="{a4db4c2b-c5e8-4071-a7cd-2df124f7c271}" mentionId="{8984a4e6-8f3e-49d5-b058-f4b3f322d5a6}" startIndex="70" length="21"/>
     </x18tc:mentions>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="E73" dT="2026-06-08T13:38:54.00" personId="{96b38dae-aaad-4c58-8713-07ba69f8f13c}" id="{521d4cde-75cd-454b-b98e-61333b99ef39}" parentId="{f06b32da-dd55-4e63-aef3-1f65e72a0c83}">
+  <x18tc:threadedComment ref="E73" dT="2026-06-08T13:38:54.00" personId="{18a4e096-09dc-487e-94e2-bb4f2bc6690b}" id="{f4b5fff5-84a7-450b-b5b5-21ec6fe520f4}" parentId="{bbd46d50-5793-4f27-acbb-bf2b066df97a}">
     <x18tc:text xml:space="preserve">Apenas o valor relativo à obra = R$ 1.000,00</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="E68" dT="2026-06-03T21:29:16.00" personId="{96b38dae-aaad-4c58-8713-07ba69f8f13c}" id="{2a7dcfa7-c60f-45b9-842b-040baa35e254}" done="1">
+  <x18tc:threadedComment ref="E68" dT="2026-06-03T21:29:16.00" personId="{18a4e096-09dc-487e-94e2-bb4f2bc6690b}" id="{8244c2f2-4132-4074-9ca2-389a2fe912cd}" done="1">
     <x18tc:text xml:space="preserve">Verificar esse valor, pelo QDD esse Projeto/Atividade só computa R$ 47.042.981,28 @luisalnr@gmail.com</x18tc:text>
     <x18tc:mentions>
-      <x18tc:mention mentionpersonId="{412111f0-d9ef-41f6-b055-45c4ed45d33c}" mentionId="{90f250da-d5e6-4196-b946-647c4ebac419}" startIndex="82" length="19"/>
+      <x18tc:mention mentionpersonId="{04d0802d-6b46-4da0-9c28-31ea27299ecf}" mentionId="{29d4e9f1-e002-40bc-a4e0-b0e90847866a}" startIndex="82" length="19"/>
     </x18tc:mentions>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="E68" dT="2026-06-08T12:59:46.00" personId="{4a970b55-9de4-44b4-b664-773b73a5c0ca}" id="{17afef39-fefd-4e38-a3d5-af6658c0a1cb}" parentId="{2a7dcfa7-c60f-45b9-842b-040baa35e254}">
+  <x18tc:threadedComment ref="E68" dT="2026-06-08T12:59:46.00" personId="{85e82f82-b122-4a5e-827e-e13eb07226b3}" id="{e341b169-42c0-476c-bcb0-2345d3c7983a}" parentId="{8244c2f2-4132-4074-9ca2-389a2fe912cd}">
     <x18tc:text xml:space="preserve">De acordo com o SICAF, é este valor mesmo de R$ 97.285.647,31</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A73" dT="2026-06-05T13:55:13.00" personId="{96b38dae-aaad-4c58-8713-07ba69f8f13c}" id="{c04e08d9-b3a5-458c-a077-712e51e5ccf6}" done="1">
+  <x18tc:threadedComment ref="A73" dT="2026-06-05T13:55:13.00" personId="{18a4e096-09dc-487e-94e2-bb4f2bc6690b}" id="{3db4590b-99b0-46f9-8e5c-535b09fd0c09}" done="1">
     <x18tc:text xml:space="preserve">Não apareceram os seguintes órgãos: TCE, TJAC, DPE, MPAC (estão listados na planilha anterior, mas não estão nesta) @luisalnr@gmail.com
 Assigned to luisalnr@gmail.com</x18tc:text>
     <x18tc:mentions>
-      <x18tc:mention mentionpersonId="{412111f0-d9ef-41f6-b055-45c4ed45d33c}" mentionId="{d1cca60a-a306-4c14-ba9a-197043d694a9}" startIndex="116" length="19"/>
+      <x18tc:mention mentionpersonId="{04d0802d-6b46-4da0-9c28-31ea27299ecf}" mentionId="{f8e03a6e-ccfb-401d-8bf0-1a9122dca0e4}" startIndex="116" length="19"/>
     </x18tc:mentions>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-06-03T18:33:29.00" personId="{96b38dae-aaad-4c58-8713-07ba69f8f13c}" id="{0619dc93-171c-4da2-b441-412af1ac3113}" done="1">
+  <x18tc:threadedComment ref="A1" dT="2026-06-03T18:33:29.00" personId="{18a4e096-09dc-487e-94e2-bb4f2bc6690b}" id="{8ba3ea41-de65-44d7-bcaf-e66d12b358bb}" done="1">
     <x18tc:text xml:space="preserve">@luisalnr@gmail.com manter apenas no Eixo VI - linha 163 da planilha</x18tc:text>
     <x18tc:mentions>
-      <x18tc:mention mentionpersonId="{412111f0-d9ef-41f6-b055-45c4ed45d33c}" mentionId="{942a7798-e932-4ddc-b0dd-143a787fd7f2}" startIndex="0" length="19"/>
+      <x18tc:mention mentionpersonId="{04d0802d-6b46-4da0-9c28-31ea27299ecf}" mentionId="{a71f5bba-37ab-4118-abfb-9c82b953353b}" startIndex="0" length="19"/>
     </x18tc:mentions>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -3523,7 +3517,7 @@
         <v>121.0</v>
       </c>
       <c r="D74" s="21" t="s">
-        <v>104</v>
+        <v>10</v>
       </c>
       <c r="E74" s="28">
         <v>2.0E7</v>
@@ -3532,7 +3526,7 @@
         <v>2.228E7</v>
       </c>
       <c r="G74" s="23" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H74" s="29" t="s">
         <v>45</v>
@@ -3549,7 +3543,7 @@
         <v>122.0</v>
       </c>
       <c r="D75" s="34" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E75" s="38">
         <v>100000.0</v>
@@ -3558,7 +3552,7 @@
         <v>2.152E7</v>
       </c>
       <c r="G75" s="36" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H75" s="29" t="s">
         <v>45</v>
@@ -3575,7 +3569,7 @@
         <v>122.0</v>
       </c>
       <c r="D76" s="34" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E76" s="35">
         <f>50000+60000</f>
@@ -3585,7 +3579,7 @@
         <v>2.12E7</v>
       </c>
       <c r="G76" s="36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H76" s="29" t="s">
         <v>45</v>
@@ -3611,7 +3605,7 @@
         <v>1.197E7</v>
       </c>
       <c r="G77" s="36" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H77" s="29" t="s">
         <v>45</v>
@@ -3637,13 +3631,10 @@
         <v>1.199E7</v>
       </c>
       <c r="G78" s="36" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H78" s="29" t="s">
         <v>45</v>
-      </c>
-      <c r="I78" s="39">
-        <v>4.0</v>
       </c>
     </row>
     <row r="79">
@@ -3666,7 +3657,7 @@
         <v>1.203E7</v>
       </c>
       <c r="G79" s="36" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H79" s="29" t="s">
         <v>45</v>
@@ -3692,7 +3683,7 @@
         <v>1.204E7</v>
       </c>
       <c r="G80" s="36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H80" s="29" t="s">
         <v>45</v>
@@ -3718,7 +3709,7 @@
         <v>2.221E7</v>
       </c>
       <c r="G81" s="36" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H81" s="29" t="s">
         <v>45</v>
@@ -3735,7 +3726,7 @@
         <v>129.0</v>
       </c>
       <c r="D82" s="34" t="s">
-        <v>104</v>
+        <v>10</v>
       </c>
       <c r="E82" s="38">
         <v>1000000.0</v>
@@ -3744,7 +3735,7 @@
         <v>1.197E7</v>
       </c>
       <c r="G82" s="36" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H82" s="29" t="s">
         <v>45</v>
@@ -3761,7 +3752,7 @@
         <v>129.0</v>
       </c>
       <c r="D83" s="34" t="s">
-        <v>104</v>
+        <v>10</v>
       </c>
       <c r="E83" s="38">
         <v>4000000.0</v>
@@ -3770,7 +3761,7 @@
         <v>1.203E7</v>
       </c>
       <c r="G83" s="36" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H83" s="29" t="s">
         <v>45</v>
@@ -3781,7 +3772,7 @@
         <v>100</v>
       </c>
       <c r="B84" s="32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C84" s="37">
         <v>181.0</v>
@@ -3796,7 +3787,7 @@
         <v>1.365E7</v>
       </c>
       <c r="G84" s="36" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H84" s="29" t="s">
         <v>45</v>
@@ -3807,13 +3798,13 @@
         <v>100</v>
       </c>
       <c r="B85" s="32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C85" s="37">
         <v>182.0</v>
       </c>
       <c r="D85" s="34" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E85" s="35">
         <v>1000.0</v>
@@ -3822,7 +3813,7 @@
         <v>1.015E7</v>
       </c>
       <c r="G85" s="36" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H85" s="29" t="s">
         <v>45</v>
@@ -3833,13 +3824,13 @@
         <v>100</v>
       </c>
       <c r="B86" s="32" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C86" s="37">
         <v>182.0</v>
       </c>
       <c r="D86" s="34" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E86" s="38">
         <v>500000.0</v>
@@ -3848,7 +3839,7 @@
         <v>1.012E7</v>
       </c>
       <c r="G86" s="36" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H86" s="29" t="s">
         <v>45</v>
@@ -3859,13 +3850,13 @@
         <v>100</v>
       </c>
       <c r="B87" s="32" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C87" s="37">
         <v>182.0</v>
       </c>
       <c r="D87" s="34" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E87" s="38">
         <v>1999000.0</v>
@@ -3874,7 +3865,7 @@
         <v>1.014E7</v>
       </c>
       <c r="G87" s="36" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H87" s="29" t="s">
         <v>45</v>
@@ -3885,13 +3876,13 @@
         <v>100</v>
       </c>
       <c r="B88" s="32" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C88" s="33">
         <v>183.0</v>
       </c>
       <c r="D88" s="34" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E88" s="38">
         <v>200000.0</v>
@@ -3900,7 +3891,7 @@
         <v>2.075E7</v>
       </c>
       <c r="G88" s="36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H88" s="29" t="s">
         <v>45</v>
@@ -3911,13 +3902,13 @@
         <v>100</v>
       </c>
       <c r="B89" s="32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C89" s="37">
         <v>183.0</v>
       </c>
       <c r="D89" s="34" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E89" s="35">
         <v>3300000.0</v>
@@ -3926,7 +3917,7 @@
         <v>1.105E7</v>
       </c>
       <c r="G89" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H89" s="29" t="s">
         <v>45</v>
@@ -3937,13 +3928,13 @@
         <v>100</v>
       </c>
       <c r="B90" s="19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C90" s="20">
         <v>183.0</v>
       </c>
       <c r="D90" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E90" s="28">
         <v>800.0</v>
@@ -3952,7 +3943,7 @@
         <v>1.093E7</v>
       </c>
       <c r="G90" s="23" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H90" s="29" t="s">
         <v>45</v>
@@ -3963,7 +3954,7 @@
         <v>100</v>
       </c>
       <c r="B91" s="32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C91" s="37">
         <v>183.0</v>
@@ -3971,7 +3962,7 @@
       <c r="D91" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="E91" s="40">
+      <c r="E91" s="39">
         <f>600000+3700000</f>
         <v>4300000</v>
       </c>
@@ -3979,7 +3970,7 @@
         <v>1.116E7</v>
       </c>
       <c r="G91" s="36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H91" s="29" t="s">
         <v>45</v>
@@ -3990,13 +3981,13 @@
         <v>100</v>
       </c>
       <c r="B92" s="19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C92" s="20">
         <v>183.0</v>
       </c>
       <c r="D92" s="21" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E92" s="22">
         <v>1771713.29</v>
@@ -4005,7 +3996,7 @@
         <v>1.093E7</v>
       </c>
       <c r="G92" s="23" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H92" s="29" t="s">
         <v>45</v>
@@ -4016,7 +4007,7 @@
         <v>100</v>
       </c>
       <c r="B93" s="32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C93" s="37">
         <v>183.0</v>
@@ -4024,7 +4015,7 @@
       <c r="D93" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="E93" s="40">
+      <c r="E93" s="39">
         <f>2800000</f>
         <v>2800000</v>
       </c>
@@ -4032,7 +4023,7 @@
         <v>1.116E7</v>
       </c>
       <c r="G93" s="36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H93" s="29" t="s">
         <v>45</v>
@@ -4043,7 +4034,7 @@
         <v>100</v>
       </c>
       <c r="B94" s="32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C94" s="37">
         <v>183.0</v>
@@ -4051,14 +4042,14 @@
       <c r="D94" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="E94" s="41">
+      <c r="E94" s="40">
         <v>50000.0</v>
       </c>
       <c r="F94" s="36">
         <v>1.115E7</v>
       </c>
       <c r="G94" s="36" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H94" s="29" t="s">
         <v>45</v>
@@ -4069,7 +4060,7 @@
         <v>100</v>
       </c>
       <c r="B95" s="32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C95" s="33">
         <v>183.0</v>
@@ -4077,14 +4068,14 @@
       <c r="D95" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="E95" s="41">
+      <c r="E95" s="40">
         <v>250000.0</v>
       </c>
       <c r="F95" s="36">
         <v>1.112E7</v>
       </c>
       <c r="G95" s="36" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H95" s="29" t="s">
         <v>45</v>
@@ -4095,7 +4086,7 @@
         <v>100</v>
       </c>
       <c r="B96" s="32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C96" s="33">
         <v>183.0</v>
@@ -4103,14 +4094,14 @@
       <c r="D96" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="E96" s="41">
+      <c r="E96" s="40">
         <v>400000.0</v>
       </c>
       <c r="F96" s="36">
         <v>1.115E7</v>
       </c>
       <c r="G96" s="36" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H96" s="29" t="s">
         <v>45</v>
@@ -4121,13 +4112,13 @@
         <v>100</v>
       </c>
       <c r="B97" s="32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C97" s="37">
         <v>183.0</v>
       </c>
       <c r="D97" s="34" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E97" s="35">
         <f>3300000</f>
@@ -4137,7 +4128,7 @@
         <v>1.022E7</v>
       </c>
       <c r="G97" s="36" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H97" s="29" t="s">
         <v>45</v>
@@ -4147,23 +4138,23 @@
       <c r="A98" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="B98" s="42" t="s">
-        <v>119</v>
+      <c r="B98" s="41" t="s">
+        <v>118</v>
       </c>
       <c r="C98" s="37">
         <v>183.0</v>
       </c>
       <c r="D98" s="34" t="s">
-        <v>133</v>
-      </c>
-      <c r="E98" s="41">
+        <v>132</v>
+      </c>
+      <c r="E98" s="40">
         <v>1000000.0</v>
       </c>
       <c r="F98" s="36">
         <v>2.076E7</v>
       </c>
       <c r="G98" s="36" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H98" s="29" t="s">
         <v>45</v>
@@ -4174,13 +4165,13 @@
         <v>100</v>
       </c>
       <c r="B99" s="32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C99" s="37">
         <v>421.0</v>
       </c>
       <c r="D99" s="34" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E99" s="35">
         <v>1000000.0</v>
@@ -4189,7 +4180,7 @@
         <v>1.09E7</v>
       </c>
       <c r="G99" s="36" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H99" s="29" t="s">
         <v>45</v>
@@ -4200,7 +4191,7 @@
         <v>100</v>
       </c>
       <c r="B100" s="32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C100" s="37">
         <v>542.0</v>
@@ -4226,13 +4217,13 @@
         <v>100</v>
       </c>
       <c r="B101" s="32" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C101" s="37">
         <v>122.0</v>
       </c>
       <c r="D101" s="34" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E101" s="35">
         <v>1000.0</v>
@@ -4241,7 +4232,7 @@
         <v>2.251E7</v>
       </c>
       <c r="G101" s="36" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H101" s="29" t="s">
         <v>45</v>
@@ -4252,13 +4243,13 @@
         <v>100</v>
       </c>
       <c r="B102" s="19" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C102" s="20">
         <v>244.0</v>
       </c>
       <c r="D102" s="21" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E102" s="28">
         <v>5000000.0</v>
@@ -4267,7 +4258,7 @@
         <v>1.221E7</v>
       </c>
       <c r="G102" s="23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H102" s="29" t="s">
         <v>45</v>
@@ -4278,22 +4269,22 @@
         <v>100</v>
       </c>
       <c r="B103" s="32" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C103" s="37">
         <v>122.0</v>
       </c>
       <c r="D103" s="34" t="s">
-        <v>142</v>
-      </c>
-      <c r="E103" s="41">
+        <v>141</v>
+      </c>
+      <c r="E103" s="40">
         <v>100000.0</v>
       </c>
       <c r="F103" s="36">
         <v>2.019E7</v>
       </c>
       <c r="G103" s="36" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H103" s="29" t="s">
         <v>45</v>
@@ -4304,13 +4295,13 @@
         <v>100</v>
       </c>
       <c r="B104" s="19" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C104" s="20">
         <v>272.0</v>
       </c>
       <c r="D104" s="21" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E104" s="28">
         <v>4000000.0</v>
@@ -4319,7 +4310,7 @@
         <v>2.021E7</v>
       </c>
       <c r="G104" s="23" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H104" s="29" t="s">
         <v>45</v>
@@ -4330,15 +4321,15 @@
         <v>100</v>
       </c>
       <c r="B105" s="32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C105" s="37">
         <v>302.0</v>
       </c>
       <c r="D105" s="34" t="s">
-        <v>146</v>
-      </c>
-      <c r="E105" s="40">
+        <v>145</v>
+      </c>
+      <c r="E105" s="39">
         <f>44510000</f>
         <v>44510000</v>
       </c>
@@ -4346,7 +4337,7 @@
         <v>1.173E7</v>
       </c>
       <c r="G105" s="36" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H105" s="29" t="s">
         <v>45</v>
@@ -4357,13 +4348,13 @@
         <v>100</v>
       </c>
       <c r="B106" s="32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C106" s="37">
         <v>302.0</v>
       </c>
       <c r="D106" s="34" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E106" s="38">
         <v>1.2997E7</v>
@@ -4372,7 +4363,7 @@
         <v>2.208E7</v>
       </c>
       <c r="G106" s="36" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H106" s="29" t="s">
         <v>45</v>
@@ -4383,15 +4374,15 @@
         <v>100</v>
       </c>
       <c r="B107" s="32" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C107" s="37">
         <v>695.0</v>
       </c>
       <c r="D107" s="34" t="s">
-        <v>150</v>
-      </c>
-      <c r="E107" s="40">
+        <v>149</v>
+      </c>
+      <c r="E107" s="39">
         <f>700000+1</f>
         <v>700001</v>
       </c>
@@ -4399,7 +4390,7 @@
         <v>1.151E7</v>
       </c>
       <c r="G107" s="36" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H107" s="29" t="s">
         <v>45</v>
@@ -4410,13 +4401,13 @@
         <v>100</v>
       </c>
       <c r="B108" s="32" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C108" s="37">
         <v>695.0</v>
       </c>
       <c r="D108" s="34" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E108" s="38">
         <v>1.0</v>
@@ -4425,7 +4416,7 @@
         <v>1152000.0</v>
       </c>
       <c r="G108" s="36" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H108" s="29" t="s">
         <v>12</v>
@@ -4436,13 +4427,13 @@
         <v>100</v>
       </c>
       <c r="B109" s="32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C109" s="37">
         <v>361.0</v>
       </c>
       <c r="D109" s="34" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E109" s="38">
         <v>1900000.0</v>
@@ -4451,7 +4442,7 @@
         <v>2.089E7</v>
       </c>
       <c r="G109" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H109" s="29" t="s">
         <v>45</v>
@@ -4462,13 +4453,13 @@
         <v>100</v>
       </c>
       <c r="B110" s="32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C110" s="37">
         <v>361.0</v>
       </c>
       <c r="D110" s="34" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E110" s="38">
         <v>2.495E7</v>
@@ -4477,7 +4468,7 @@
         <v>1.041E7</v>
       </c>
       <c r="G110" s="36" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H110" s="29" t="s">
         <v>45</v>
@@ -4488,13 +4479,13 @@
         <v>100</v>
       </c>
       <c r="B111" s="32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C111" s="37">
         <v>362.0</v>
       </c>
       <c r="D111" s="34" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E111" s="35">
         <f>4000000</f>
@@ -4504,7 +4495,7 @@
         <v>1.04E7</v>
       </c>
       <c r="G111" s="36" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H111" s="29" t="s">
         <v>45</v>
@@ -4515,13 +4506,13 @@
         <v>100</v>
       </c>
       <c r="B112" s="32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C112" s="37">
         <v>363.0</v>
       </c>
       <c r="D112" s="34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E112" s="38">
         <v>500.0</v>
@@ -4530,7 +4521,7 @@
         <v>2.082E7</v>
       </c>
       <c r="G112" s="36" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H112" s="29" t="s">
         <v>45</v>
@@ -4541,13 +4532,13 @@
         <v>100</v>
       </c>
       <c r="B113" s="32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C113" s="37">
         <v>363.0</v>
       </c>
       <c r="D113" s="34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E113" s="38">
         <v>500.0</v>
@@ -4556,7 +4547,7 @@
         <v>1.025E7</v>
       </c>
       <c r="G113" s="36" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H113" s="29" t="s">
         <v>45</v>
@@ -4567,13 +4558,13 @@
         <v>100</v>
       </c>
       <c r="B114" s="32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C114" s="37">
         <v>363.0</v>
       </c>
       <c r="D114" s="34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E114" s="38">
         <v>1601000.0</v>
@@ -4582,7 +4573,7 @@
         <v>1.023E7</v>
       </c>
       <c r="G114" s="36" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H114" s="29" t="s">
         <v>45</v>
@@ -4593,13 +4584,13 @@
         <v>100</v>
       </c>
       <c r="B115" s="32" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C115" s="37">
         <v>122.0</v>
       </c>
       <c r="D115" s="36" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E115" s="38">
         <v>147472.27</v>
@@ -4608,7 +4599,7 @@
         <v>1.299E7</v>
       </c>
       <c r="G115" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H115" s="29" t="s">
         <v>45</v>
@@ -4619,13 +4610,13 @@
         <v>100</v>
       </c>
       <c r="B116" s="32" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C116" s="37">
         <v>122.0</v>
       </c>
       <c r="D116" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E116" s="38">
         <v>151000.0</v>
@@ -4634,7 +4625,7 @@
         <v>1.299E7</v>
       </c>
       <c r="G116" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H116" s="29" t="s">
         <v>45</v>
@@ -4645,13 +4636,13 @@
         <v>100</v>
       </c>
       <c r="B117" s="32" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C117" s="33">
         <v>392.0</v>
       </c>
       <c r="D117" s="34" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E117" s="38">
         <v>750000.0</v>
@@ -4660,7 +4651,7 @@
         <v>1.29E7</v>
       </c>
       <c r="G117" s="36" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H117" s="29" t="s">
         <v>45</v>
@@ -4671,13 +4662,13 @@
         <v>100</v>
       </c>
       <c r="B118" s="32" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C118" s="33">
         <v>392.0</v>
       </c>
       <c r="D118" s="34" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E118" s="38">
         <v>290000.0</v>
@@ -4686,7 +4677,7 @@
         <v>1.292E7</v>
       </c>
       <c r="G118" s="36" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H118" s="29" t="s">
         <v>45</v>
@@ -4697,13 +4688,13 @@
         <v>100</v>
       </c>
       <c r="B119" s="32" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C119" s="37">
         <v>243.0</v>
       </c>
       <c r="D119" s="34" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E119" s="35">
         <v>2251384.93</v>
@@ -4712,7 +4703,7 @@
         <v>1.011E7</v>
       </c>
       <c r="G119" s="36" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H119" s="29" t="s">
         <v>45</v>
@@ -4723,13 +4714,13 @@
         <v>100</v>
       </c>
       <c r="B120" s="19" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C120" s="20">
         <v>422.0</v>
       </c>
       <c r="D120" s="21" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E120" s="28">
         <v>5000.0</v>
@@ -4738,7 +4729,7 @@
         <v>1.036E7</v>
       </c>
       <c r="G120" s="23" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H120" s="29" t="s">
         <v>45</v>
@@ -4749,13 +4740,13 @@
         <v>100</v>
       </c>
       <c r="B121" s="32" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C121" s="37">
         <v>422.0</v>
       </c>
       <c r="D121" s="34" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E121" s="35">
         <v>589560.0</v>
@@ -4764,7 +4755,7 @@
         <v>1.147E7</v>
       </c>
       <c r="G121" s="36" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H121" s="29" t="s">
         <v>45</v>
@@ -4775,13 +4766,13 @@
         <v>100</v>
       </c>
       <c r="B122" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C122" s="37">
         <v>451.0</v>
       </c>
       <c r="D122" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E122" s="38">
         <v>1000.0</v>
@@ -4790,7 +4781,7 @@
         <v>1.058E7</v>
       </c>
       <c r="G122" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H122" s="29" t="s">
         <v>12</v>
@@ -4801,13 +4792,13 @@
         <v>100</v>
       </c>
       <c r="B123" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C123" s="37">
         <v>451.0</v>
       </c>
       <c r="D123" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E123" s="38">
         <v>9362139.29</v>
@@ -4816,7 +4807,7 @@
         <v>1.059E7</v>
       </c>
       <c r="G123" s="36" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H123" s="29" t="s">
         <v>12</v>
@@ -4827,13 +4818,13 @@
         <v>100</v>
       </c>
       <c r="B124" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C124" s="37">
         <v>451.0</v>
       </c>
       <c r="D124" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E124" s="38">
         <v>3.49143533E7</v>
@@ -4842,7 +4833,7 @@
         <v>1.06E7</v>
       </c>
       <c r="G124" s="36" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H124" s="29" t="s">
         <v>45</v>
@@ -4853,13 +4844,13 @@
         <v>100</v>
       </c>
       <c r="B125" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C125" s="37">
         <v>451.0</v>
       </c>
       <c r="D125" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E125" s="38">
         <v>1001000.0</v>
@@ -4868,7 +4859,7 @@
         <v>1.061E7</v>
       </c>
       <c r="G125" s="36" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H125" s="29" t="s">
         <v>45</v>
@@ -4879,13 +4870,13 @@
         <v>100</v>
       </c>
       <c r="B126" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C126" s="37">
         <v>451.0</v>
       </c>
       <c r="D126" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E126" s="38">
         <v>1000.0</v>
@@ -4894,7 +4885,7 @@
         <v>1.34E7</v>
       </c>
       <c r="G126" s="36" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H126" s="29" t="s">
         <v>45</v>
@@ -4905,13 +4896,13 @@
         <v>100</v>
       </c>
       <c r="B127" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C127" s="37">
         <v>451.0</v>
       </c>
       <c r="D127" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E127" s="38">
         <v>1000.0</v>
@@ -4920,7 +4911,7 @@
         <v>2.306E7</v>
       </c>
       <c r="G127" s="36" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H127" s="29" t="s">
         <v>45</v>
@@ -4931,7 +4922,7 @@
         <v>100</v>
       </c>
       <c r="B128" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C128" s="37">
         <v>451.0</v>
@@ -4946,7 +4937,7 @@
         <v>1.099E7</v>
       </c>
       <c r="G128" s="36" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H128" s="29" t="s">
         <v>12</v>
@@ -4957,7 +4948,7 @@
         <v>100</v>
       </c>
       <c r="B129" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C129" s="37">
         <v>451.0</v>
@@ -4972,7 +4963,7 @@
         <v>2.201E7</v>
       </c>
       <c r="G129" s="36" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H129" s="29" t="s">
         <v>45</v>
@@ -4983,13 +4974,13 @@
         <v>100</v>
       </c>
       <c r="B130" s="19" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C130" s="20">
         <v>451.0</v>
       </c>
       <c r="D130" s="21" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E130" s="28">
         <v>1000.0</v>
@@ -4998,7 +4989,7 @@
         <v>1.059E7</v>
       </c>
       <c r="G130" s="23" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H130" s="29" t="s">
         <v>12</v>
@@ -5009,13 +5000,13 @@
         <v>100</v>
       </c>
       <c r="B131" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C131" s="37">
         <v>451.0</v>
       </c>
       <c r="D131" s="34" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E131" s="38">
         <v>1.78625E7</v>
@@ -5024,7 +5015,7 @@
         <v>1.097E7</v>
       </c>
       <c r="G131" s="36" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H131" s="29" t="s">
         <v>45</v>
@@ -5035,13 +5026,13 @@
         <v>100</v>
       </c>
       <c r="B132" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C132" s="37">
         <v>451.0</v>
       </c>
       <c r="D132" s="34" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E132" s="38">
         <v>9938000.0</v>
@@ -5050,7 +5041,7 @@
         <v>1.098E7</v>
       </c>
       <c r="G132" s="36" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H132" s="29" t="s">
         <v>45</v>
@@ -5061,13 +5052,13 @@
         <v>100</v>
       </c>
       <c r="B133" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C133" s="37">
         <v>451.0</v>
       </c>
       <c r="D133" s="34" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E133" s="38">
         <f>4800000+3600000+9000000</f>
@@ -5077,7 +5068,7 @@
         <v>1.099E7</v>
       </c>
       <c r="G133" s="36" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H133" s="29" t="s">
         <v>12</v>
@@ -5088,13 +5079,13 @@
         <v>100</v>
       </c>
       <c r="B134" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C134" s="37">
         <v>451.0</v>
       </c>
       <c r="D134" s="34" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E134" s="38">
         <v>5705000.0</v>
@@ -5103,7 +5094,7 @@
         <v>1.1E7</v>
       </c>
       <c r="G134" s="36" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H134" s="29" t="s">
         <v>45</v>
@@ -5114,13 +5105,13 @@
         <v>100</v>
       </c>
       <c r="B135" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C135" s="37">
         <v>451.0</v>
       </c>
       <c r="D135" s="34" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E135" s="38">
         <v>1.0E7</v>
@@ -5129,7 +5120,7 @@
         <v>1.331E7</v>
       </c>
       <c r="G135" s="36" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H135" s="29" t="s">
         <v>45</v>
@@ -5140,13 +5131,13 @@
         <v>100</v>
       </c>
       <c r="B136" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C136" s="37">
         <v>451.0</v>
       </c>
       <c r="D136" s="34" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E136" s="38">
         <v>1.6034E7</v>
@@ -5155,7 +5146,7 @@
         <v>2.142E7</v>
       </c>
       <c r="G136" s="36" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H136" s="29" t="s">
         <v>45</v>
@@ -5166,15 +5157,15 @@
         <v>100</v>
       </c>
       <c r="B137" s="32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C137" s="37">
         <v>512.0</v>
       </c>
       <c r="D137" s="34" t="s">
-        <v>176</v>
-      </c>
-      <c r="E137" s="40">
+        <v>175</v>
+      </c>
+      <c r="E137" s="39">
         <f>3000</f>
         <v>3000</v>
       </c>
@@ -5182,7 +5173,7 @@
         <v>1.337E7</v>
       </c>
       <c r="G137" s="36" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H137" s="29" t="s">
         <v>45</v>
@@ -5193,13 +5184,13 @@
         <v>100</v>
       </c>
       <c r="B138" s="32" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C138" s="37">
         <v>122.0</v>
       </c>
       <c r="D138" s="34" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E138" s="38">
         <v>150000.0</v>
@@ -5208,7 +5199,7 @@
         <v>2.275E7</v>
       </c>
       <c r="G138" s="36" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H138" s="29" t="s">
         <v>45</v>
@@ -5219,13 +5210,13 @@
         <v>100</v>
       </c>
       <c r="B139" s="19" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C139" s="20">
         <v>482.0</v>
       </c>
       <c r="D139" s="21" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E139" s="28">
         <v>100000.0</v>
@@ -5234,7 +5225,7 @@
         <v>1.057E7</v>
       </c>
       <c r="G139" s="23" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H139" s="29" t="s">
         <v>45</v>
@@ -5245,22 +5236,22 @@
         <v>100</v>
       </c>
       <c r="B140" s="32" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C140" s="37">
         <v>482.0</v>
       </c>
       <c r="D140" s="34" t="s">
-        <v>176</v>
-      </c>
-      <c r="E140" s="41">
+        <v>175</v>
+      </c>
+      <c r="E140" s="40">
         <v>7541842.2</v>
       </c>
       <c r="F140" s="36">
         <v>1.057E7</v>
       </c>
       <c r="G140" s="36" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H140" s="29" t="s">
         <v>45</v>
@@ -5271,13 +5262,13 @@
         <v>100</v>
       </c>
       <c r="B141" s="32" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C141" s="37">
         <v>512.0</v>
       </c>
       <c r="D141" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E141" s="38">
         <v>3000.0</v>
@@ -5286,7 +5277,7 @@
         <v>1.338E7</v>
       </c>
       <c r="G141" s="36" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H141" s="29" t="s">
         <v>45</v>
@@ -5297,13 +5288,13 @@
         <v>100</v>
       </c>
       <c r="B142" s="19" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C142" s="20">
         <v>512.0</v>
       </c>
       <c r="D142" s="21" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E142" s="22">
         <v>3221000.0</v>
@@ -5312,7 +5303,7 @@
         <v>1.101E7</v>
       </c>
       <c r="G142" s="23" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H142" s="29" t="s">
         <v>45</v>
@@ -5323,13 +5314,13 @@
         <v>100</v>
       </c>
       <c r="B143" s="19" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C143" s="20">
         <v>512.0</v>
       </c>
       <c r="D143" s="21" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E143" s="22">
         <v>1000000.0</v>
@@ -5338,7 +5329,7 @@
         <v>1.102E7</v>
       </c>
       <c r="G143" s="23" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H143" s="29" t="s">
         <v>45</v>
@@ -5349,13 +5340,13 @@
         <v>100</v>
       </c>
       <c r="B144" s="19" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C144" s="20">
         <v>512.0</v>
       </c>
       <c r="D144" s="21" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E144" s="22">
         <v>8550000.0</v>
@@ -5364,7 +5355,7 @@
         <v>1.103E7</v>
       </c>
       <c r="G144" s="23" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H144" s="29" t="s">
         <v>45</v>
@@ -5375,7 +5366,7 @@
         <v>100</v>
       </c>
       <c r="B145" s="32" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C145" s="37">
         <v>512.0</v>
@@ -5390,7 +5381,7 @@
         <v>1.129E7</v>
       </c>
       <c r="G145" s="36" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H145" s="29" t="s">
         <v>45</v>
@@ -5401,7 +5392,7 @@
         <v>100</v>
       </c>
       <c r="B146" s="32" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C146" s="37">
         <v>512.0</v>
@@ -5416,7 +5407,7 @@
         <v>1130000.0</v>
       </c>
       <c r="G146" s="36" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H146" s="29" t="s">
         <v>45</v>
@@ -5427,7 +5418,7 @@
         <v>100</v>
       </c>
       <c r="B147" s="19" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C147" s="20">
         <v>512.0</v>
@@ -5442,7 +5433,7 @@
         <v>1.045E7</v>
       </c>
       <c r="G147" s="23" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H147" s="29" t="s">
         <v>45</v>
@@ -5494,7 +5485,7 @@
         <v>1.138E7</v>
       </c>
       <c r="G149" s="23" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H149" s="29" t="s">
         <v>45</v>
@@ -5505,13 +5496,13 @@
         <v>100</v>
       </c>
       <c r="B150" s="32" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C150" s="37">
         <v>571.0</v>
       </c>
       <c r="D150" s="34" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E150" s="35">
         <v>10.0</v>
@@ -5520,7 +5511,7 @@
         <v>1.156E7</v>
       </c>
       <c r="G150" s="36" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H150" s="29" t="s">
         <v>45</v>
@@ -5546,7 +5537,7 @@
         <v>1.084E7</v>
       </c>
       <c r="G151" s="23" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H151" s="29" t="s">
         <v>45</v>
@@ -5563,7 +5554,7 @@
         <v>451.0</v>
       </c>
       <c r="D152" s="34" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E152" s="35">
         <v>2000000.0</v>
@@ -5572,7 +5563,7 @@
         <v>1.073E7</v>
       </c>
       <c r="G152" s="36" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H152" s="29" t="s">
         <v>45</v>
@@ -5636,13 +5627,13 @@
         <v>100</v>
       </c>
       <c r="B155" s="32" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C155" s="37">
         <v>127.0</v>
       </c>
       <c r="D155" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E155" s="38">
         <v>1000.0</v>
@@ -5651,7 +5642,7 @@
         <v>1.339E7</v>
       </c>
       <c r="G155" s="36" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H155" s="29" t="s">
         <v>45</v>
@@ -5662,7 +5653,7 @@
         <v>100</v>
       </c>
       <c r="B156" s="32" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C156" s="37">
         <v>122.0</v>
@@ -5677,7 +5668,7 @@
         <v>2.203E7</v>
       </c>
       <c r="G156" s="36" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H156" s="29" t="s">
         <v>45</v>
@@ -5688,7 +5679,7 @@
         <v>100</v>
       </c>
       <c r="B157" s="32" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C157" s="37">
         <v>451.0</v>
@@ -5703,7 +5694,7 @@
         <v>1.171E7</v>
       </c>
       <c r="G157" s="36" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H157" s="29" t="s">
         <v>45</v>
@@ -5714,7 +5705,7 @@
         <v>100</v>
       </c>
       <c r="B158" s="32" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C158" s="37">
         <v>781.0</v>
@@ -5729,7 +5720,7 @@
         <v>1.168E7</v>
       </c>
       <c r="G158" s="36" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H158" s="29" t="s">
         <v>45</v>
@@ -5740,7 +5731,7 @@
         <v>100</v>
       </c>
       <c r="B159" s="32" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C159" s="37">
         <v>782.0</v>
@@ -5755,7 +5746,7 @@
         <v>1.169E7</v>
       </c>
       <c r="G159" s="36" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H159" s="29" t="s">
         <v>45</v>
@@ -5766,7 +5757,7 @@
         <v>100</v>
       </c>
       <c r="B160" s="32" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C160" s="37">
         <v>782.0</v>
@@ -5781,7 +5772,7 @@
         <v>2.196E7</v>
       </c>
       <c r="G160" s="36" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H160" s="29" t="s">
         <v>45</v>
@@ -5792,7 +5783,7 @@
         <v>100</v>
       </c>
       <c r="B161" s="32" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C161" s="37">
         <v>782.0</v>
@@ -5807,7 +5798,7 @@
         <v>2.197E7</v>
       </c>
       <c r="G161" s="36" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H161" s="29" t="s">
         <v>45</v>
@@ -5818,7 +5809,7 @@
         <v>100</v>
       </c>
       <c r="B162" s="32" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C162" s="37">
         <v>782.0</v>
@@ -5833,7 +5824,7 @@
         <v>2.198E7</v>
       </c>
       <c r="G162" s="36" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H162" s="29" t="s">
         <v>45</v>
@@ -5844,7 +5835,7 @@
         <v>100</v>
       </c>
       <c r="B163" s="32" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C163" s="37">
         <v>782.0</v>
@@ -5859,7 +5850,7 @@
         <v>2.199E7</v>
       </c>
       <c r="G163" s="36" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H163" s="29" t="s">
         <v>45</v>
@@ -5870,7 +5861,7 @@
         <v>100</v>
       </c>
       <c r="B164" s="32" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C164" s="37">
         <v>782.0</v>
@@ -5885,7 +5876,7 @@
         <v>2.2E7</v>
       </c>
       <c r="G164" s="36" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H164" s="29" t="s">
         <v>45</v>
@@ -5896,13 +5887,13 @@
         <v>100</v>
       </c>
       <c r="B165" s="32" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C165" s="37">
         <v>812.0</v>
       </c>
       <c r="D165" s="34" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E165" s="35">
         <v>4466051.73</v>
@@ -5911,14 +5902,14 @@
         <v>1.332E7</v>
       </c>
       <c r="G165" s="36" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H165" s="29" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="166">
-      <c r="F166" s="43"/>
+      <c r="F166" s="42"/>
       <c r="G166" s="18"/>
       <c r="H166" s="18"/>
     </row>
@@ -5948,16 +5939,16 @@
     </row>
     <row r="168">
       <c r="A168" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="B168" s="19" t="s">
         <v>226</v>
-      </c>
-      <c r="B168" s="19" t="s">
-        <v>227</v>
       </c>
       <c r="C168" s="20">
         <v>244.0</v>
       </c>
       <c r="D168" s="21" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E168" s="22">
         <v>79000.0</v>
@@ -5966,7 +5957,7 @@
         <v>1.222E7</v>
       </c>
       <c r="G168" s="23" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H168" s="25" t="s">
         <v>45</v>
@@ -5974,16 +5965,16 @@
     </row>
     <row r="169">
       <c r="A169" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="B169" s="19" t="s">
         <v>226</v>
-      </c>
-      <c r="B169" s="19" t="s">
-        <v>227</v>
       </c>
       <c r="C169" s="20">
         <v>244.0</v>
       </c>
       <c r="D169" s="21" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E169" s="22">
         <v>1000000.0</v>
@@ -5992,7 +5983,7 @@
         <v>1.236E7</v>
       </c>
       <c r="G169" s="23" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H169" s="25" t="s">
         <v>45</v>
@@ -6000,16 +5991,16 @@
     </row>
     <row r="170">
       <c r="A170" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="B170" s="19" t="s">
         <v>226</v>
-      </c>
-      <c r="B170" s="19" t="s">
-        <v>227</v>
       </c>
       <c r="C170" s="20">
         <v>244.0</v>
       </c>
       <c r="D170" s="21" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E170" s="22">
         <v>69000.0</v>
@@ -6018,7 +6009,7 @@
         <v>1.254E7</v>
       </c>
       <c r="G170" s="23" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H170" s="25" t="s">
         <v>45</v>
@@ -6026,16 +6017,16 @@
     </row>
     <row r="171">
       <c r="A171" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="B171" s="19" t="s">
         <v>226</v>
-      </c>
-      <c r="B171" s="19" t="s">
-        <v>227</v>
       </c>
       <c r="C171" s="20">
         <v>244.0</v>
       </c>
       <c r="D171" s="21" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E171" s="22">
         <v>800000.0</v>
@@ -6044,7 +6035,7 @@
         <v>1.266E7</v>
       </c>
       <c r="G171" s="23" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H171" s="25" t="s">
         <v>12</v>
@@ -6052,16 +6043,16 @@
     </row>
     <row r="172">
       <c r="A172" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="B172" s="19" t="s">
         <v>226</v>
-      </c>
-      <c r="B172" s="19" t="s">
-        <v>227</v>
       </c>
       <c r="C172" s="20">
         <v>244.0</v>
       </c>
       <c r="D172" s="21" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E172" s="22">
         <v>529000.0</v>
@@ -6070,7 +6061,7 @@
         <v>1.249E7</v>
       </c>
       <c r="G172" s="23" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H172" s="29" t="s">
         <v>12</v>
@@ -6078,16 +6069,16 @@
     </row>
     <row r="173">
       <c r="A173" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="B173" s="19" t="s">
         <v>226</v>
-      </c>
-      <c r="B173" s="19" t="s">
-        <v>227</v>
       </c>
       <c r="C173" s="20">
         <v>244.0</v>
       </c>
       <c r="D173" s="21" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E173" s="22">
         <v>50000.0</v>
@@ -6096,7 +6087,7 @@
         <v>1.266E7</v>
       </c>
       <c r="G173" s="23" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H173" s="29" t="s">
         <v>12</v>
@@ -6104,16 +6095,16 @@
     </row>
     <row r="174">
       <c r="A174" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B174" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C174" s="20">
         <v>422.0</v>
       </c>
       <c r="D174" s="21" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E174" s="28">
         <v>65200.0</v>
@@ -6122,7 +6113,7 @@
         <v>1.043E7</v>
       </c>
       <c r="G174" s="23" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H174" s="25" t="s">
         <v>45</v>
@@ -6130,16 +6121,16 @@
     </row>
     <row r="175">
       <c r="A175" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B175" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C175" s="20">
         <v>422.0</v>
       </c>
       <c r="D175" s="21" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E175" s="28">
         <v>580000.0</v>
@@ -6148,7 +6139,7 @@
         <v>1.223E7</v>
       </c>
       <c r="G175" s="23" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H175" s="25" t="s">
         <v>45</v>
@@ -6156,16 +6147,16 @@
     </row>
     <row r="176">
       <c r="A176" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B176" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C176" s="20">
         <v>422.0</v>
       </c>
       <c r="D176" s="21" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E176" s="22">
         <v>178000.0</v>
@@ -6174,7 +6165,7 @@
         <v>1.027E7</v>
       </c>
       <c r="G176" s="23" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H176" s="25" t="s">
         <v>45</v>
@@ -6182,16 +6173,16 @@
     </row>
     <row r="177">
       <c r="A177" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B177" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C177" s="20">
         <v>422.0</v>
       </c>
       <c r="D177" s="21" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E177" s="22">
         <v>71000.0</v>
@@ -6200,7 +6191,7 @@
         <v>1.028E7</v>
       </c>
       <c r="G177" s="23" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H177" s="25" t="s">
         <v>45</v>
@@ -6208,16 +6199,16 @@
     </row>
     <row r="178">
       <c r="A178" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B178" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C178" s="20">
         <v>422.0</v>
       </c>
       <c r="D178" s="21" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E178" s="22">
         <v>321000.0</v>
@@ -6226,7 +6217,7 @@
         <v>1.029E7</v>
       </c>
       <c r="G178" s="23" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H178" s="25" t="s">
         <v>45</v>
@@ -6234,16 +6225,16 @@
     </row>
     <row r="179">
       <c r="A179" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B179" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C179" s="20">
         <v>422.0</v>
       </c>
       <c r="D179" s="21" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E179" s="22">
         <v>221000.0</v>
@@ -6252,7 +6243,7 @@
         <v>1.03E7</v>
       </c>
       <c r="G179" s="23" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H179" s="25" t="s">
         <v>45</v>
@@ -6260,16 +6251,16 @@
     </row>
     <row r="180">
       <c r="A180" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B180" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C180" s="20">
         <v>422.0</v>
       </c>
       <c r="D180" s="21" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E180" s="22">
         <v>4048000.0</v>
@@ -6278,7 +6269,7 @@
         <v>2.083E7</v>
       </c>
       <c r="G180" s="23" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H180" s="25" t="s">
         <v>45</v>
@@ -6286,16 +6277,16 @@
     </row>
     <row r="181">
       <c r="A181" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B181" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C181" s="20">
         <v>422.0</v>
       </c>
       <c r="D181" s="21" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E181" s="28">
         <v>1030000.0</v>
@@ -6304,7 +6295,7 @@
         <v>1.035E7</v>
       </c>
       <c r="G181" s="23" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H181" s="25" t="s">
         <v>45</v>
@@ -6312,16 +6303,16 @@
     </row>
     <row r="182">
       <c r="A182" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B182" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C182" s="20">
         <v>422.0</v>
       </c>
       <c r="D182" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E182" s="28">
         <f>2415560-1937560</f>
@@ -6331,7 +6322,7 @@
         <v>1.146E7</v>
       </c>
       <c r="G182" s="23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H182" s="25" t="s">
         <v>45</v>
@@ -6339,16 +6330,16 @@
     </row>
     <row r="183">
       <c r="A183" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B183" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C183" s="20">
         <v>423.0</v>
       </c>
       <c r="D183" s="21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E183" s="22">
         <v>2000.0</v>
@@ -6357,7 +6348,7 @@
         <v>1.086E7</v>
       </c>
       <c r="G183" s="23" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H183" s="29" t="s">
         <v>12</v>
@@ -6365,16 +6356,16 @@
     </row>
     <row r="184">
       <c r="A184" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B184" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C184" s="20">
         <v>423.0</v>
       </c>
       <c r="D184" s="21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E184" s="22">
         <v>2000.0</v>
@@ -6383,7 +6374,7 @@
         <v>1.087E7</v>
       </c>
       <c r="G184" s="23" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H184" s="29" t="s">
         <v>12</v>
@@ -6391,16 +6382,16 @@
     </row>
     <row r="185">
       <c r="A185" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B185" s="19" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C185" s="20">
         <v>127.0</v>
       </c>
       <c r="D185" s="21" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E185" s="28">
         <v>1151000.0</v>
@@ -6409,7 +6400,7 @@
         <v>1.339E7</v>
       </c>
       <c r="G185" s="23" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H185" s="25" t="s">
         <v>45</v>
@@ -6417,16 +6408,16 @@
     </row>
     <row r="186">
       <c r="A186" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B186" s="19" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C186" s="20">
         <v>127.0</v>
       </c>
       <c r="D186" s="21" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E186" s="22">
         <v>797700.0</v>
@@ -6435,7 +6426,7 @@
         <v>1.031E7</v>
       </c>
       <c r="G186" s="23" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H186" s="25" t="s">
         <v>45</v>
@@ -6443,16 +6434,16 @@
     </row>
     <row r="187">
       <c r="A187" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B187" s="19" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C187" s="20">
         <v>127.0</v>
       </c>
       <c r="D187" s="21" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E187" s="22">
         <v>5156900.0</v>
@@ -6461,7 +6452,7 @@
         <v>1.032E7</v>
       </c>
       <c r="G187" s="23" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H187" s="25" t="s">
         <v>45</v>
@@ -6469,16 +6460,16 @@
     </row>
     <row r="188">
       <c r="A188" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B188" s="19" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C188" s="20">
         <v>127.0</v>
       </c>
       <c r="D188" s="21" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E188" s="22">
         <v>102000.0</v>
@@ -6487,7 +6478,7 @@
         <v>1.033E7</v>
       </c>
       <c r="G188" s="23" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H188" s="25" t="s">
         <v>45</v>
@@ -6495,16 +6486,16 @@
     </row>
     <row r="189">
       <c r="A189" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B189" s="19" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C189" s="20">
         <v>127.0</v>
       </c>
       <c r="D189" s="21" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E189" s="22">
         <v>20000.0</v>
@@ -6513,7 +6504,7 @@
         <v>1.034E7</v>
       </c>
       <c r="G189" s="23" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H189" s="25" t="s">
         <v>45</v>
@@ -6521,16 +6512,16 @@
     </row>
     <row r="190">
       <c r="A190" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B190" s="19" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C190" s="20">
         <v>127.0</v>
       </c>
       <c r="D190" s="21" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E190" s="22">
         <v>6110535.52</v>
@@ -6539,7 +6530,7 @@
         <v>2.084E7</v>
       </c>
       <c r="G190" s="23" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H190" s="25" t="s">
         <v>45</v>
@@ -6578,16 +6569,16 @@
     </row>
     <row r="193">
       <c r="A193" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="B193" s="19" t="s">
         <v>252</v>
-      </c>
-      <c r="B193" s="19" t="s">
-        <v>253</v>
       </c>
       <c r="C193" s="20">
         <v>124.0</v>
       </c>
       <c r="D193" s="21" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E193" s="28">
         <v>660000.0</v>
@@ -6596,15 +6587,15 @@
         <v>1.085E7</v>
       </c>
       <c r="G193" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="H193" s="44" t="s">
+        <v>254</v>
+      </c>
+      <c r="H193" s="43" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="19" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B194" s="19" t="s">
         <v>9</v>
@@ -6621,16 +6612,16 @@
       <c r="F194" s="23">
         <v>1.126E7</v>
       </c>
-      <c r="G194" s="45" t="s">
+      <c r="G194" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="H194" s="44" t="s">
+      <c r="H194" s="43" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="19" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B195" s="19" t="s">
         <v>9</v>
@@ -6647,10 +6638,10 @@
       <c r="F195" s="23">
         <v>1.141E7</v>
       </c>
-      <c r="G195" s="45" t="s">
-        <v>256</v>
-      </c>
-      <c r="H195" s="44" t="s">
+      <c r="G195" s="44" t="s">
+        <v>255</v>
+      </c>
+      <c r="H195" s="43" t="s">
         <v>12</v>
       </c>
     </row>
@@ -6687,7 +6678,7 @@
     </row>
     <row r="198">
       <c r="A198" s="19" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B198" s="19" t="s">
         <v>73</v>
@@ -6713,7 +6704,7 @@
     </row>
     <row r="199">
       <c r="A199" s="19" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B199" s="19" t="s">
         <v>73</v>
@@ -6739,16 +6730,16 @@
     </row>
     <row r="200">
       <c r="A200" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="B200" s="19" t="s">
         <v>257</v>
-      </c>
-      <c r="B200" s="19" t="s">
-        <v>258</v>
       </c>
       <c r="C200" s="20">
         <v>571.0</v>
       </c>
       <c r="D200" s="21" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E200" s="28">
         <v>60.0</v>
@@ -6757,7 +6748,7 @@
         <v>1.156E7</v>
       </c>
       <c r="G200" s="23" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H200" s="25" t="s">
         <v>12</v>
@@ -6765,16 +6756,16 @@
     </row>
     <row r="201">
       <c r="A201" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="B201" s="19" t="s">
         <v>257</v>
-      </c>
-      <c r="B201" s="19" t="s">
-        <v>258</v>
       </c>
       <c r="C201" s="20">
         <v>573.0</v>
       </c>
       <c r="D201" s="21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E201" s="22">
         <v>1156486.0</v>
@@ -6783,7 +6774,7 @@
         <v>1.219E7</v>
       </c>
       <c r="G201" s="23" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="H201" s="25" t="s">
         <v>12</v>
@@ -6791,16 +6782,16 @@
     </row>
     <row r="202">
       <c r="A202" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="B202" s="19" t="s">
         <v>257</v>
-      </c>
-      <c r="B202" s="19" t="s">
-        <v>258</v>
       </c>
       <c r="C202" s="20">
         <v>573.0</v>
       </c>
       <c r="D202" s="21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E202" s="22">
         <v>1.0</v>
@@ -6809,7 +6800,7 @@
         <v>1.22E7</v>
       </c>
       <c r="G202" s="23" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="H202" s="25" t="s">
         <v>12</v>
@@ -6817,16 +6808,16 @@
     </row>
     <row r="203">
       <c r="A203" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="B203" s="19" t="s">
         <v>257</v>
-      </c>
-      <c r="B203" s="19" t="s">
-        <v>258</v>
       </c>
       <c r="C203" s="20">
         <v>573.0</v>
       </c>
       <c r="D203" s="21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E203" s="22">
         <v>1.0</v>
@@ -6835,7 +6826,7 @@
         <v>1.278E7</v>
       </c>
       <c r="G203" s="23" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="H203" s="25" t="s">
         <v>12</v>
@@ -6843,16 +6834,16 @@
     </row>
     <row r="204">
       <c r="A204" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="B204" s="19" t="s">
         <v>257</v>
-      </c>
-      <c r="B204" s="19" t="s">
-        <v>258</v>
       </c>
       <c r="C204" s="20">
         <v>573.0</v>
       </c>
       <c r="D204" s="21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E204" s="22">
         <v>2.0</v>
@@ -6861,7 +6852,7 @@
         <v>1.28E7</v>
       </c>
       <c r="G204" s="23" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H204" s="25" t="s">
         <v>12</v>
@@ -6869,10 +6860,10 @@
     </row>
     <row r="205">
       <c r="A205" s="19" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B205" s="19" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C205" s="20">
         <v>573.0</v>
@@ -6887,7 +6878,7 @@
         <v>1.341E7</v>
       </c>
       <c r="G205" s="23" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="H205" s="25" t="s">
         <v>12</v>
@@ -6895,10 +6886,10 @@
     </row>
     <row r="206">
       <c r="A206" s="19" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B206" s="19" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C206" s="20">
         <v>573.0</v>
@@ -6913,7 +6904,7 @@
         <v>1.342E7</v>
       </c>
       <c r="G206" s="23" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="H206" s="25" t="s">
         <v>12</v>
@@ -6921,10 +6912,10 @@
     </row>
     <row r="207">
       <c r="A207" s="19" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B207" s="19" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C207" s="20">
         <v>573.0</v>
@@ -6939,7 +6930,7 @@
         <v>1.343E7</v>
       </c>
       <c r="G207" s="23" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="H207" s="25" t="s">
         <v>12</v>
@@ -6947,16 +6938,16 @@
     </row>
     <row r="208">
       <c r="A208" s="19" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B208" s="19" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C208" s="20">
         <v>573.0</v>
       </c>
       <c r="D208" s="21" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E208" s="28">
         <v>700050.0</v>
@@ -6965,7 +6956,7 @@
         <v>1.158E7</v>
       </c>
       <c r="G208" s="23" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="H208" s="25" t="s">
         <v>12</v>
@@ -7004,16 +6995,16 @@
     </row>
     <row r="211">
       <c r="A211" s="19" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B211" s="19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C211" s="20">
         <v>182.0</v>
       </c>
       <c r="D211" s="21" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E211" s="22">
         <v>4000.0</v>
@@ -7021,8 +7012,8 @@
       <c r="F211" s="23">
         <v>1.013E7</v>
       </c>
-      <c r="G211" s="46" t="s">
-        <v>270</v>
+      <c r="G211" s="45" t="s">
+        <v>269</v>
       </c>
       <c r="H211" s="25" t="s">
         <v>12</v>
@@ -7030,16 +7021,16 @@
     </row>
     <row r="212">
       <c r="A212" s="19" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B212" s="19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C212" s="20">
         <v>182.0</v>
       </c>
       <c r="D212" s="21" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E212" s="22">
         <v>589667.0</v>
@@ -7047,8 +7038,8 @@
       <c r="F212" s="23">
         <v>2.272E7</v>
       </c>
-      <c r="G212" s="46" t="s">
-        <v>271</v>
+      <c r="G212" s="45" t="s">
+        <v>270</v>
       </c>
       <c r="H212" s="25" t="s">
         <v>12</v>
@@ -7056,16 +7047,16 @@
     </row>
     <row r="213">
       <c r="A213" s="19" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B213" s="19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C213" s="20">
         <v>182.0</v>
       </c>
       <c r="D213" s="21" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E213" s="28">
         <v>1.7753E7</v>
@@ -7073,8 +7064,8 @@
       <c r="F213" s="23">
         <v>2.079E7</v>
       </c>
-      <c r="G213" s="46" t="s">
-        <v>272</v>
+      <c r="G213" s="45" t="s">
+        <v>271</v>
       </c>
       <c r="H213" s="25" t="s">
         <v>12</v>
@@ -7082,16 +7073,16 @@
     </row>
     <row r="214">
       <c r="A214" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="B214" s="19" t="s">
         <v>226</v>
-      </c>
-      <c r="B214" s="19" t="s">
-        <v>227</v>
       </c>
       <c r="C214" s="20">
         <v>244.0</v>
       </c>
       <c r="D214" s="21" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E214" s="28">
         <v>250000.0</v>
@@ -7099,15 +7090,15 @@
       <c r="F214" s="23">
         <v>1.242E7</v>
       </c>
-      <c r="G214" s="46" t="s">
-        <v>273</v>
-      </c>
-      <c r="H214" s="47" t="s">
+      <c r="G214" s="45" t="s">
+        <v>272</v>
+      </c>
+      <c r="H214" s="46" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="215">
-      <c r="F215" s="48"/>
+      <c r="F215" s="47"/>
     </row>
   </sheetData>
   <dataValidations>

</xml_diff>